<commit_message>
Validate household taxonomy semantics and human package
</commit_message>
<xml_diff>
--- a/taxonomies/open-household-records-taxonomy/taxonomy.xlsx
+++ b/taxonomies/open-household-records-taxonomy/taxonomy.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>home or tenant policy • vehicle policy • life policy • travel policy • claim record • proof of insurance • renewal notice</t>
+          <t>home or tenant policy • vehicle policy • life policy • travel policy • pet insurance policy • claim record • proof of insurance • renewal notice</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Home &amp; property • Vehicles &amp; transportation • Health &amp; care • Travel • Financial</t>
+          <t>Home &amp; property • Vehicles &amp; transportation • Health &amp; care • Travel • Financial • Pets</t>
         </is>
       </c>
     </row>
@@ -908,17 +908,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>School, childcare, activity, enrolment, permission, progress, and other records primarily connected to a child's education or organized activities.</t>
+          <t>Records connected to education, training, childcare, children's activities, enrolment, permission, progress, and related learning or dependant administration.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>school enrolment record • report card • permission form • childcare information • activity registration • school notice • pickup or release instruction</t>
+          <t>school or post-secondary enrolment record • report card or transcript • diploma or certificate • permission form • childcare information • activity registration • school notice • pickup or release instruction</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Use only where children, dependants, education, childcare, or youth activities are relevant to the household.</t>
+          <t>Use for education or training records that household members keep, and for child or dependant records whose primary purpose is school, childcare, activities, or related administration.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>new school, childcare, or program • new academic or activity period • contact or pickup arrangement change • custody or guardian change • health or accommodation change • child ages out or record loses practical relevance</t>
+          <t>new school, course, training, childcare, or program • new academic or activity period • completion, graduation, or credential issue • contact or pickup arrangement change • custody or guardian change • health or accommodation change • record loses practical relevance</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -982,27 +982,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Veterinary, vaccination, registration, insurance, medication, adoption, licence, and care records associated with household animals.</t>
+          <t>Veterinary, vaccination, registration, medication, adoption, licence, and care records associated with household animals.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>veterinary record • vaccination record • prescription • pet insurance • licence • adoption record • microchip information • care instruction</t>
+          <t>veterinary record • vaccination record • prescription • licence • adoption record • microchip information • care instruction • boarding or caregiver record</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Use where the household has animals whose health, ownership, care, registration, or insurance information is worth maintaining.</t>
+          <t>Use where the household has animals whose health, ownership, care, registration, or practical care information is worth maintaining.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Depends on the record: Pet records are often low-risk, but owner contact details, addresses, payment information, access arrangements, or insurance information can increase sensitivity.</t>
+          <t>Depends on the record: Pet records are often low-risk, but owner contact details, addresses, payment information, access arrangements, or care information can increase sensitivity.</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>adoption or ownership change • veterinarian change • medication or care change • vaccination or licence update • insurance change • pet lost, rehomed, or deceased</t>
+          <t>adoption or ownership change • veterinarian change • medication or care change • vaccination or licence update • pet lost, rehomed, or deceased</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Trip-specific bookings, visas, itineraries, insurance, confirmations, rentals, and supporting travel information.</t>
+          <t>Trip-specific bookings, visas, itineraries, confirmations, rentals, and supporting travel information.</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>flight or rail booking • hotel confirmation • visa • travel insurance • itinerary • rental agreement • tour or activity confirmation</t>
+          <t>flight or rail booking • hotel confirmation • visa • itinerary • rental agreement • tour or activity confirmation • refund or cancellation record</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>booking or itinerary change • visa or entry-document change • travel insurance change • trip cancelled or completed • claim, refund, or dispute • travel document expires</t>
+          <t>booking or itinerary change • visa or entry-document change • trip cancelled or completed • claim, refund, or dispute • travel document expires</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1092,132 +1092,6 @@
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Open Household Records Taxonomy</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Human-readable workbook — Public Review Candidate v0.1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="45" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Core rule</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Give each record one primary category based on what it is mainly about. Keep other useful connections as relationships or references rather than making competing copies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Quick test</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>If this record disappeared, which part of household life would notice first? That is usually the best clue to its primary category.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>What this is</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>A practical reference for classifying household records across paper folders, cloud storage, spreadsheets, software, or AI-assisted tools.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>What this is not</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>It is not a legal, tax, medical, insurance, privacy, security, or retention standard. A category existing does not mean every household must have records in it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Sensitivity labels</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>These are practical handling cues only. They are not legal classifications.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Review triggers</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Examples of life or record changes that should prompt somebody to check whether information is still current or useful.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Machine files</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>The companion CSV, JSON, and JSON Schema exist for portability and software use. This workbook is the human-facing spreadsheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Public Review Candidate v0.1.0. Reuse licensing remains intentionally unresolved until founder review.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1335,7 +1209,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>ohrt.home_property | ohrt.vehicles_transportation | ohrt.health_care | ohrt.travel | ohrt.financial</t>
+          <t>ohrt.home_property | ohrt.vehicles_transportation | ohrt.health_care | ohrt.travel | ohrt.financial | ohrt.pets</t>
         </is>
       </c>
     </row>

</xml_diff>